<commit_message>
actualizar excels - 2026-06-05 20:14
</commit_message>
<xml_diff>
--- a/op_det_os.xlsx
+++ b/op_det_os.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,76 +413,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N917"/>
+  <dimension ref="A1:N940"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Num-OP</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>OP Det</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cantidad OP-D</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Detalle</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Cliente</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Total Precio</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Id_OS</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Cantidad OS</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Servicio</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Num OS</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Fecha OS</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Fecha Op-Det</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Id op-det</t>
         </is>
@@ -50479,6 +50467,1202 @@
         <v>86330323</v>
       </c>
     </row>
+    <row r="918">
+      <c r="A918" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>6832-1-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C918" t="n">
+        <v>1</v>
+      </c>
+      <c r="D918" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y ESPALDA  FILTRO GRUPO  B</t>
+        </is>
+      </c>
+      <c r="E918" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F918" t="n">
+        <v>70888</v>
+      </c>
+      <c r="G918" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H918" t="inlineStr"/>
+      <c r="I918" t="inlineStr"/>
+      <c r="J918" t="inlineStr"/>
+      <c r="K918" t="inlineStr"/>
+      <c r="L918" t="inlineStr"/>
+      <c r="M918" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N918" t="n">
+        <v>86341650</v>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>6832-2-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C919" t="n">
+        <v>1</v>
+      </c>
+      <c r="D919" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y  ESPALDA  FILTRO GRUPO  A</t>
+        </is>
+      </c>
+      <c r="E919" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F919" t="n">
+        <v>70888</v>
+      </c>
+      <c r="G919" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H919" t="inlineStr"/>
+      <c r="I919" t="inlineStr"/>
+      <c r="J919" t="inlineStr"/>
+      <c r="K919" t="inlineStr"/>
+      <c r="L919" t="inlineStr"/>
+      <c r="M919" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N919" t="n">
+        <v>86341674</v>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>6832-3-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C920" t="n">
+        <v>1</v>
+      </c>
+      <c r="D920" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y ESPALDA RECURSOS HUMANOS</t>
+        </is>
+      </c>
+      <c r="E920" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F920" t="n">
+        <v>70888</v>
+      </c>
+      <c r="G920" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H920" t="inlineStr"/>
+      <c r="I920" t="inlineStr"/>
+      <c r="J920" t="inlineStr"/>
+      <c r="K920" t="inlineStr"/>
+      <c r="L920" t="inlineStr"/>
+      <c r="M920" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N920" t="n">
+        <v>86341698</v>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>6832-4-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C921" t="n">
+        <v>1</v>
+      </c>
+      <c r="D921" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y  ESPALDA LIDER LYD</t>
+        </is>
+      </c>
+      <c r="E921" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F921" t="n">
+        <v>70888</v>
+      </c>
+      <c r="G921" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H921" t="inlineStr"/>
+      <c r="I921" t="inlineStr"/>
+      <c r="J921" t="inlineStr"/>
+      <c r="K921" t="inlineStr"/>
+      <c r="L921" t="inlineStr"/>
+      <c r="M921" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N921" t="n">
+        <v>86341722</v>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>6832-5-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C922" t="n">
+        <v>1</v>
+      </c>
+      <c r="D922" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y  ESPALDA LIDER DESPACHO B</t>
+        </is>
+      </c>
+      <c r="E922" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F922" t="n">
+        <v>70888</v>
+      </c>
+      <c r="G922" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H922" t="inlineStr"/>
+      <c r="I922" t="inlineStr"/>
+      <c r="J922" t="inlineStr"/>
+      <c r="K922" t="inlineStr"/>
+      <c r="L922" t="inlineStr"/>
+      <c r="M922" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N922" t="n">
+        <v>86341746</v>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>6832-6-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C923" t="n">
+        <v>1</v>
+      </c>
+      <c r="D923" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y ESPALDA LIDER DESPACHO  A</t>
+        </is>
+      </c>
+      <c r="E923" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F923" t="n">
+        <v>70888</v>
+      </c>
+      <c r="G923" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H923" t="inlineStr"/>
+      <c r="I923" t="inlineStr"/>
+      <c r="J923" t="inlineStr"/>
+      <c r="K923" t="inlineStr"/>
+      <c r="L923" t="inlineStr"/>
+      <c r="M923" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N923" t="n">
+        <v>86341771</v>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>6832-7-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C924" t="n">
+        <v>2</v>
+      </c>
+      <c r="D924" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y ESPALDA TUNELERO GRUPO B</t>
+        </is>
+      </c>
+      <c r="E924" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F924" t="n">
+        <v>141776</v>
+      </c>
+      <c r="G924" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H924" t="inlineStr"/>
+      <c r="I924" t="inlineStr"/>
+      <c r="J924" t="inlineStr"/>
+      <c r="K924" t="inlineStr"/>
+      <c r="L924" t="inlineStr"/>
+      <c r="M924" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N924" t="n">
+        <v>86341795</v>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>6832-8-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C925" t="n">
+        <v>2</v>
+      </c>
+      <c r="D925" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y   ESPALDA TUNELERO GRUPO A</t>
+        </is>
+      </c>
+      <c r="E925" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F925" t="n">
+        <v>141776</v>
+      </c>
+      <c r="G925" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H925" t="inlineStr"/>
+      <c r="I925" t="inlineStr"/>
+      <c r="J925" t="inlineStr"/>
+      <c r="K925" t="inlineStr"/>
+      <c r="L925" t="inlineStr"/>
+      <c r="M925" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N925" t="n">
+        <v>86341821</v>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>6832-9-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C926" t="n">
+        <v>1</v>
+      </c>
+      <c r="D926" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y    ESPALDA SALMUERA GRUPO B</t>
+        </is>
+      </c>
+      <c r="E926" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F926" t="n">
+        <v>70888</v>
+      </c>
+      <c r="G926" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H926" t="inlineStr"/>
+      <c r="I926" t="inlineStr"/>
+      <c r="J926" t="inlineStr"/>
+      <c r="K926" t="inlineStr"/>
+      <c r="L926" t="inlineStr"/>
+      <c r="M926" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N926" t="n">
+        <v>86341845</v>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>6832-10-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C927" t="n">
+        <v>1</v>
+      </c>
+      <c r="D927" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y   ESPALDA SALMUERA GRUPO A</t>
+        </is>
+      </c>
+      <c r="E927" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F927" t="n">
+        <v>70888</v>
+      </c>
+      <c r="G927" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H927" t="inlineStr"/>
+      <c r="I927" t="inlineStr"/>
+      <c r="J927" t="inlineStr"/>
+      <c r="K927" t="inlineStr"/>
+      <c r="L927" t="inlineStr"/>
+      <c r="M927" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N927" t="n">
+        <v>86341869</v>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>6832-11-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C928" t="n">
+        <v>3</v>
+      </c>
+      <c r="D928" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y   ESPALDA DESPRECE MANUAL B</t>
+        </is>
+      </c>
+      <c r="E928" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F928" t="n">
+        <v>212664</v>
+      </c>
+      <c r="G928" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H928" t="inlineStr"/>
+      <c r="I928" t="inlineStr"/>
+      <c r="J928" t="inlineStr"/>
+      <c r="K928" t="inlineStr"/>
+      <c r="L928" t="inlineStr"/>
+      <c r="M928" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N928" t="n">
+        <v>86341893</v>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>6832-12-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C929" t="n">
+        <v>3</v>
+      </c>
+      <c r="D929" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y   ESPALDA DESPRECE MANUAL A</t>
+        </is>
+      </c>
+      <c r="E929" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F929" t="n">
+        <v>212664</v>
+      </c>
+      <c r="G929" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H929" t="inlineStr"/>
+      <c r="I929" t="inlineStr"/>
+      <c r="J929" t="inlineStr"/>
+      <c r="K929" t="inlineStr"/>
+      <c r="L929" t="inlineStr"/>
+      <c r="M929" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N929" t="n">
+        <v>86341919</v>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>6832-13-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C930" t="n">
+        <v>1</v>
+      </c>
+      <c r="D930" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y   ESPALDA LIDER DESPRECE MANUAL B</t>
+        </is>
+      </c>
+      <c r="E930" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F930" t="n">
+        <v>70888</v>
+      </c>
+      <c r="G930" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H930" t="inlineStr"/>
+      <c r="I930" t="inlineStr"/>
+      <c r="J930" t="inlineStr"/>
+      <c r="K930" t="inlineStr"/>
+      <c r="L930" t="inlineStr"/>
+      <c r="M930" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N930" t="n">
+        <v>86341943</v>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>6832-14-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C931" t="n">
+        <v>1</v>
+      </c>
+      <c r="D931" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y   ESPALDA LIDER DESPRECE MANUAL A</t>
+        </is>
+      </c>
+      <c r="E931" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F931" t="n">
+        <v>70888</v>
+      </c>
+      <c r="G931" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H931" t="inlineStr"/>
+      <c r="I931" t="inlineStr"/>
+      <c r="J931" t="inlineStr"/>
+      <c r="K931" t="inlineStr"/>
+      <c r="L931" t="inlineStr"/>
+      <c r="M931" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N931" t="n">
+        <v>86341967</v>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>6832-15-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C932" t="n">
+        <v>3</v>
+      </c>
+      <c r="D932" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y   ESPALDA SUPERVISOR PRODUCCION</t>
+        </is>
+      </c>
+      <c r="E932" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F932" t="n">
+        <v>212664</v>
+      </c>
+      <c r="G932" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H932" t="inlineStr"/>
+      <c r="I932" t="inlineStr"/>
+      <c r="J932" t="inlineStr"/>
+      <c r="K932" t="inlineStr"/>
+      <c r="L932" t="inlineStr"/>
+      <c r="M932" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N932" t="n">
+        <v>86341991</v>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>6832-16-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C933" t="n">
+        <v>6</v>
+      </c>
+      <c r="D933" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y   ESPALDA LIDER PRODUCCION</t>
+        </is>
+      </c>
+      <c r="E933" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F933" t="n">
+        <v>425328</v>
+      </c>
+      <c r="G933" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H933" t="inlineStr"/>
+      <c r="I933" t="inlineStr"/>
+      <c r="J933" t="inlineStr"/>
+      <c r="K933" t="inlineStr"/>
+      <c r="L933" t="inlineStr"/>
+      <c r="M933" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N933" t="n">
+        <v>86342016</v>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>6832-17-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C934" t="n">
+        <v>1</v>
+      </c>
+      <c r="D934" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y   ESPALDA LIDER RECIBO B</t>
+        </is>
+      </c>
+      <c r="E934" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F934" t="n">
+        <v>70888</v>
+      </c>
+      <c r="G934" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H934" t="inlineStr"/>
+      <c r="I934" t="inlineStr"/>
+      <c r="J934" t="inlineStr"/>
+      <c r="K934" t="inlineStr"/>
+      <c r="L934" t="inlineStr"/>
+      <c r="M934" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N934" t="n">
+        <v>86342040</v>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>6832-18-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C935" t="n">
+        <v>1</v>
+      </c>
+      <c r="D935" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y  ESPALDA LIDER RECIBO A</t>
+        </is>
+      </c>
+      <c r="E935" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F935" t="n">
+        <v>70888</v>
+      </c>
+      <c r="G935" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H935" t="inlineStr"/>
+      <c r="I935" t="inlineStr"/>
+      <c r="J935" t="inlineStr"/>
+      <c r="K935" t="inlineStr"/>
+      <c r="L935" t="inlineStr"/>
+      <c r="M935" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N935" t="n">
+        <v>86342110</v>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>6832-19-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C936" t="n">
+        <v>1</v>
+      </c>
+      <c r="D936" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y  ESPALDA LIDER CUARTO FRIO B</t>
+        </is>
+      </c>
+      <c r="E936" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F936" t="n">
+        <v>70888</v>
+      </c>
+      <c r="G936" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H936" t="inlineStr"/>
+      <c r="I936" t="inlineStr"/>
+      <c r="J936" t="inlineStr"/>
+      <c r="K936" t="inlineStr"/>
+      <c r="L936" t="inlineStr"/>
+      <c r="M936" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N936" t="n">
+        <v>86342134</v>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>6832-20-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C937" t="n">
+        <v>1</v>
+      </c>
+      <c r="D937" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y  ESPALDA LIDER CUARTO FRIO A</t>
+        </is>
+      </c>
+      <c r="E937" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F937" t="n">
+        <v>70888</v>
+      </c>
+      <c r="G937" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H937" t="inlineStr"/>
+      <c r="I937" t="inlineStr"/>
+      <c r="J937" t="inlineStr"/>
+      <c r="K937" t="inlineStr"/>
+      <c r="L937" t="inlineStr"/>
+      <c r="M937" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N937" t="n">
+        <v>86342158</v>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>6832-21-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C938" t="n">
+        <v>2</v>
+      </c>
+      <c r="D938" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y  ESPALDA CUARTO GRUPO B</t>
+        </is>
+      </c>
+      <c r="E938" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F938" t="n">
+        <v>141776</v>
+      </c>
+      <c r="G938" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H938" t="inlineStr"/>
+      <c r="I938" t="inlineStr"/>
+      <c r="J938" t="inlineStr"/>
+      <c r="K938" t="inlineStr"/>
+      <c r="L938" t="inlineStr"/>
+      <c r="M938" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N938" t="n">
+        <v>86342183</v>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>6832-22-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C939" t="n">
+        <v>2</v>
+      </c>
+      <c r="D939" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y  ESPALDA CUARTO GRUPO A</t>
+        </is>
+      </c>
+      <c r="E939" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F939" t="n">
+        <v>141776</v>
+      </c>
+      <c r="G939" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H939" t="inlineStr"/>
+      <c r="I939" t="inlineStr"/>
+      <c r="J939" t="inlineStr"/>
+      <c r="K939" t="inlineStr"/>
+      <c r="L939" t="inlineStr"/>
+      <c r="M939" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N939" t="n">
+        <v>86342207</v>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="n">
+        <v>6832</v>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>6832-23-CHAQUETA SPORT</t>
+        </is>
+      </c>
+      <c r="C940" t="n">
+        <v>2</v>
+      </c>
+      <c r="D940" t="inlineStr">
+        <is>
+          <t>Chaqueta  Operativo – Unisex
+Cuello alto.
+Cierre frontal con cremallera central.
+manga larga con puño semiresortado  
+delantero liso  sin  bolsillos 
+Forro interno en  vioto 
+con  bolsillo interno tipo ribete 
+ guata acochada calibre 300
+Logo bordado en el pecho izquierdo,  y  ESPALDA AUXILIAR  REFRIGERACION</t>
+        </is>
+      </c>
+      <c r="E940" t="inlineStr">
+        <is>
+          <t>SITARA</t>
+        </is>
+      </c>
+      <c r="F940" t="n">
+        <v>141776</v>
+      </c>
+      <c r="G940" t="inlineStr">
+        <is>
+          <t>Pendiente Inicio Produccion</t>
+        </is>
+      </c>
+      <c r="H940" t="inlineStr"/>
+      <c r="I940" t="inlineStr"/>
+      <c r="J940" t="inlineStr"/>
+      <c r="K940" t="inlineStr"/>
+      <c r="L940" t="inlineStr"/>
+      <c r="M940" t="inlineStr">
+        <is>
+          <t>2026-06-05T00:22:34Z</t>
+        </is>
+      </c>
+      <c r="N940" t="n">
+        <v>86342232</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>